<commit_message>
hw 1 updated, also some other docs
</commit_message>
<xml_diff>
--- a/course_docs/PHY_905_comp_astro_tentative_schedule_Spring_2026.xlsx
+++ b/course_docs/PHY_905_comp_astro_tentative_schedule_Spring_2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bwoshea/Desktop/PHY 905 Spring 2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bwoshea/Desktop/SYNCHED/Current Projects/PHY 905 - comp astro - Spring 2026/Computational_Astro_Spring_2026/course_docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3DBEDFB-6356-A14F-BAE7-2462EF9DE832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F10705AE-7E82-5849-8C5D-FF226D26B5C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30080" yWindow="2980" windowWidth="29440" windowHeight="17820" xr2:uid="{1DD546E5-30D0-C340-B1F1-F7B464A6F5C2}"/>
   </bookViews>
@@ -158,9 +158,6 @@
     <t>Time series analysis, Part II; class wrapup.</t>
   </si>
   <si>
-    <t>Homework #1 due Friday 2/13</t>
-  </si>
-  <si>
     <t>Homework #2 due Friday 3/13</t>
   </si>
   <si>
@@ -192,6 +189,9 @@
   </si>
   <si>
     <t>May move parallel computing before Feigelson Ch. 2</t>
+  </si>
+  <si>
+    <t>Homework #1 due Sunday 2/16</t>
   </si>
 </sst>
 </file>
@@ -261,7 +261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -273,7 +273,6 @@
     <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -628,17 +627,17 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="58" customWidth="1"/>
-    <col min="5" max="5" width="39" style="13" customWidth="1"/>
+    <col min="5" max="5" width="39" style="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-      <c r="E1" s="10"/>
+      <c r="E1" s="9"/>
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -646,7 +645,7 @@
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="10"/>
+      <c r="E2" s="9"/>
       <c r="F2" s="1"/>
     </row>
     <row r="3" spans="1:6" ht="34" x14ac:dyDescent="0.2">
@@ -663,7 +662,7 @@
         <v>6</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>8</v>
@@ -682,8 +681,8 @@
       <c r="D4" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="11"/>
-      <c r="F4" s="9"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="1"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="6">
@@ -698,8 +697,8 @@
       <c r="D5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="11"/>
-      <c r="F5" s="9"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="1"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
@@ -715,7 +714,7 @@
         <v>11</v>
       </c>
       <c r="E6" s="4"/>
-      <c r="F6" s="9"/>
+      <c r="F6" s="1"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
@@ -731,7 +730,7 @@
         <v>12</v>
       </c>
       <c r="E7" s="4"/>
-      <c r="F7" s="9"/>
+      <c r="F7" s="1"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="6">
@@ -746,8 +745,8 @@
       <c r="D8" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="11"/>
-      <c r="F8" s="9"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="1"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="6">
@@ -762,8 +761,8 @@
       <c r="D9" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="12"/>
-      <c r="F9" s="9"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="1"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
@@ -779,8 +778,8 @@
         <v>15</v>
       </c>
       <c r="E10" s="4"/>
-      <c r="F10" s="9" t="s">
-        <v>49</v>
+      <c r="F10" s="1" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -797,7 +796,7 @@
         <v>16</v>
       </c>
       <c r="E11" s="4"/>
-      <c r="F11" s="9"/>
+      <c r="F11" s="1"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="6">
@@ -812,8 +811,8 @@
       <c r="D12" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E12" s="11"/>
-      <c r="F12" s="9"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="1"/>
     </row>
     <row r="13" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="6">
@@ -828,10 +827,10 @@
       <c r="D13" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="E13" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="F13" s="9"/>
+      <c r="E13" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="F13" s="1"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
@@ -847,7 +846,7 @@
         <v>34</v>
       </c>
       <c r="E14" s="4"/>
-      <c r="F14" s="9"/>
+      <c r="F14" s="1"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
@@ -863,7 +862,7 @@
         <v>19</v>
       </c>
       <c r="E15" s="4"/>
-      <c r="F15" s="9"/>
+      <c r="F15" s="1"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="6">
@@ -878,8 +877,8 @@
       <c r="D16" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E16" s="11"/>
-      <c r="F16" s="9"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="1"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="6">
@@ -894,8 +893,8 @@
       <c r="D17" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E17" s="11"/>
-      <c r="F17" s="9"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="1"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
@@ -908,8 +907,8 @@
       <c r="D18" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E18" s="10"/>
-      <c r="F18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="1"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
@@ -922,8 +921,8 @@
       <c r="D19" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E19" s="10"/>
-      <c r="F19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="1"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="6">
@@ -938,8 +937,8 @@
       <c r="D20" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E20" s="11"/>
-      <c r="F20" s="9"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="1"/>
     </row>
     <row r="21" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" s="6">
@@ -954,10 +953,10 @@
       <c r="D21" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="E21" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="F21" s="9"/>
+      <c r="E21" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="F21" s="1"/>
     </row>
     <row r="22" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
@@ -973,9 +972,9 @@
         <v>24</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="F22" s="9"/>
+        <v>43</v>
+      </c>
+      <c r="F22" s="1"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
@@ -991,7 +990,7 @@
         <v>25</v>
       </c>
       <c r="E23" s="4"/>
-      <c r="F23" s="9"/>
+      <c r="F23" s="1"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="6">
@@ -1006,9 +1005,9 @@
       <c r="D24" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E24" s="11"/>
-      <c r="F24" s="9" t="s">
-        <v>51</v>
+      <c r="E24" s="10"/>
+      <c r="F24" s="1" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
@@ -1024,8 +1023,8 @@
       <c r="D25" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E25" s="11"/>
-      <c r="F25" s="9"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="1"/>
     </row>
     <row r="26" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A26" s="3">
@@ -1041,9 +1040,9 @@
         <v>37</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="F26" s="9"/>
+        <v>44</v>
+      </c>
+      <c r="F26" s="1"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
@@ -1059,7 +1058,7 @@
         <v>26</v>
       </c>
       <c r="E27" s="4"/>
-      <c r="F27" s="9"/>
+      <c r="F27" s="1"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="6">
@@ -1074,8 +1073,8 @@
       <c r="D28" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E28" s="11"/>
-      <c r="F28" s="9"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="1"/>
     </row>
     <row r="29" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A29" s="6">
@@ -1090,10 +1089,10 @@
       <c r="D29" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E29" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="F29" s="9"/>
+      <c r="E29" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="F29" s="1"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
@@ -1109,8 +1108,8 @@
         <v>38</v>
       </c>
       <c r="E30" s="4"/>
-      <c r="F30" s="9" t="s">
-        <v>50</v>
+      <c r="F30" s="1" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1127,9 +1126,9 @@
         <v>29</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="F31" s="9"/>
+        <v>45</v>
+      </c>
+      <c r="F31" s="1"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="6">
@@ -1144,8 +1143,8 @@
       <c r="D32" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="E32" s="11"/>
-      <c r="F32" s="9"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="1"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="6">
@@ -1160,16 +1159,16 @@
       <c r="D33" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="E33" s="11"/>
-      <c r="F33" s="9"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="1"/>
     </row>
     <row r="34" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A34" s="3"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
       <c r="D34" s="1"/>
-      <c r="E34" s="10" t="s">
-        <v>43</v>
+      <c r="E34" s="9" t="s">
+        <v>42</v>
       </c>
       <c r="F34" s="1"/>
     </row>
@@ -1184,8 +1183,8 @@
       <c r="D35" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E35" s="10" t="s">
-        <v>47</v>
+      <c r="E35" s="9" t="s">
+        <v>46</v>
       </c>
       <c r="F35" s="1"/>
     </row>

</xml_diff>